<commit_message>
batch api ready for single batch
</commit_message>
<xml_diff>
--- a/data/outputs/concept_frequency_consensus.xlsx
+++ b/data/outputs/concept_frequency_consensus.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,145 +454,289 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CHW Empowered Through Training</t>
+          <t>Cholera Education and Prevention</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>claude</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>25</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CHW Empowered Through Training</t>
+          <t>Cholera Education and Prevention</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>o3</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>25</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2012</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Community Empowerment Through Education</t>
+          <t>Diabetes Education and Prevention</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>claude</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="C4" t="n">
         <v>25</v>
       </c>
       <c r="D4" t="n">
-        <v>0.672</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Community Empowerment Through Education</t>
+          <t>Diabetes Education and Prevention</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>o3</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>25</v>
       </c>
       <c r="D5" t="n">
-        <v>0.778</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Handing out Medical Supplies </t>
+          <t>Direct Intervention for Cholera Cases</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>claude</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>25</v>
       </c>
       <c r="D6" t="n">
-        <v>0.036</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Handing out Medical Supplies </t>
+          <t>Direct Intervention for Cholera Cases</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>o3</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>25</v>
       </c>
       <c r="D7" t="n">
-        <v>0.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Referrals and Advocacy</t>
+          <t>Group Based Health Education</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>claude</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>25</v>
       </c>
       <c r="D8" t="n">
-        <v>0.412</v>
+        <v>0.342</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Referrals and Advocacy</t>
+          <t>Group Based Health Education</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>o3</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>25</v>
       </c>
       <c r="D9" t="n">
-        <v>0.526</v>
+        <v>0.3488</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HIV/AIDS Education and Prevention</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.07200000000000001</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>HIV/AIDS Education and Prevention</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>25</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Individualized Support and Health Education</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>25</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.46</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Individualized Support and Health Education</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>25</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.46</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Infectious Disease Prevention</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>25</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Infectious Disease Prevention</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>25</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.384</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Tuberculosis Education and Prevention</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>25</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.052</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Tuberculosis Education and Prevention</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>25</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.07400000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -629,7 +773,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 0, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 1, 'Individualized Support and Health Education': 0, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 0, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -641,7 +785,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 1, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 0, 'Individualized Support and Health Education': 1, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 0, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -653,7 +797,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 1, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 1, 'Individualized Support and Health Education': 1, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 1, 'Tuberculosis Education and Prevention': 1}</t>
         </is>
       </c>
     </row>
@@ -665,7 +809,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 1, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 1, 'Individualized Support and Health Education': 1, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 0, 'Tuberculosis Education and Prevention': 1}</t>
         </is>
       </c>
     </row>
@@ -677,7 +821,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 1, 'Referrals and Advocacy': 0, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 0, 'Individualized Support and Health Education': 0, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 1, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -689,7 +833,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 1, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 0, 'Individualized Support and Health Education': 0, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 1, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -701,7 +845,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 1, 'Referrals and Advocacy': 1, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 0, 'Individualized Support and Health Education': 0, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 0, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -713,7 +857,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 1, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 0, 'Individualized Support and Health Education': 0, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 0, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -725,7 +869,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 1, 'Referrals and Advocacy': 1, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 1, 'Individualized Support and Health Education': 1, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 1, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -737,7 +881,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 1, 'Referrals and Advocacy': 0, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 1, 'Individualized Support and Health Education': 0, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 1, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -749,7 +893,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 1, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 1, 'Individualized Support and Health Education': 1, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 1, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -761,7 +905,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 1, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 1}</t>
+          <t>{'Group Based Health Education': 1, 'Individualized Support and Health Education': 0, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 0, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -773,7 +917,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 1, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 0, 'Individualized Support and Health Education': 1, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 1, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -785,7 +929,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 0, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 0, 'Individualized Support and Health Education': 0, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 0, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -797,7 +941,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 1, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 1, 'Individualized Support and Health Education': 1, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 1, 'Infectious Disease Prevention': 1, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -809,7 +953,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 1, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 1, 'Individualized Support and Health Education': 0, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 0, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -821,7 +965,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 1, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 0, 'Individualized Support and Health Education': 1, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 0, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -833,7 +977,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 0, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 0, 'Individualized Support and Health Education': 1, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 0, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -845,7 +989,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 0, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 0, 'Individualized Support and Health Education': 1, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 1, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 0, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -857,7 +1001,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 1, 'Community Empowerment Through Education': 0, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 0, 'Individualized Support and Health Education': 1, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 0, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -869,7 +1013,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 1, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 0, 'Individualized Support and Health Education': 0, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 1, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -881,7 +1025,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 1, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 0, 'Individualized Support and Health Education': 0, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 1, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -893,7 +1037,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 1, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 1, 'Individualized Support and Health Education': 1, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 1, 'Infectious Disease Prevention': 1, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -905,7 +1049,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 0, 'Referrals and Advocacy': 0, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 1, 'Individualized Support and Health Education': 0, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 0, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>
@@ -917,7 +1061,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>{'CHW Empowered Through Training': 1, 'Referrals and Advocacy': 1, 'Community Empowerment Through Education': 1, 'Handing out Medical Supplies ': 0}</t>
+          <t>{'Group Based Health Education': 0, 'Individualized Support and Health Education': 1, 'Cholera Education and Prevention': 0, 'Direct Intervention for Cholera Cases': 0, 'Diabetes Education and Prevention': 0, 'HIV/AIDS Education and Prevention': 0, 'Infectious Disease Prevention': 1, 'Tuberculosis Education and Prevention': 0}</t>
         </is>
       </c>
     </row>

</xml_diff>